<commit_message>
Updated build and change management files
</commit_message>
<xml_diff>
--- a/Change Management/Sample_Changes.xlsx
+++ b/Change Management/Sample_Changes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Praveen Kumar\Desktop\Git_Geeks\Change Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93F546EF-E599-4132-B3D0-69105778270A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6891DD4C-C35E-4BF4-A751-7D6066E35567}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7635" xr2:uid="{07CB3C6C-865A-4E7C-AFB0-4BDA79E1FA4D}"/>
   </bookViews>
@@ -122,16 +122,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -449,6 +452,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2344BDB7-F855-4CB8-8A79-7128175FBE4A}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="10.796875" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="12.53125" customWidth="1"/>
+    <col min="4" max="4" width="13.53125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
@@ -473,7 +482,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="57" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" s="4" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>

</xml_diff>